<commit_message>
fix(config): garrison reclaim is attack-driven, not timed — drop reclaimHours
Per the design: a player's occupied city is only lost when a hostile/neutral/third-party force
ATTACKS it (undefended -> taken directly; garrisoned -> a defense battle), symmetric to the
player taking a neutral city. It is NOT a timer, so the time-based reclaimHours field was the
wrong model — removed from the garrison table. Attack-driven reclaim belongs to a future
"enemy forces attack player cities" system. captureChance / recruitBaseRate are unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/tables/garrison.xlsx
+++ b/config/tables/garrison.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,12 +423,9 @@
         <v>leaderQuality</v>
       </c>
       <c r="H1" t="str">
-        <v>reclaimHours</v>
+        <v>captureChance</v>
       </c>
       <c r="I1" t="str">
-        <v>captureChance</v>
-      </c>
-      <c r="J1" t="str">
         <v>recruitBaseRate</v>
       </c>
     </row>
@@ -460,9 +457,6 @@
       <c r="I2">
         <v>0</v>
       </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -487,12 +481,9 @@
         <v/>
       </c>
       <c r="H3">
-        <v>24</v>
+        <v>0.25</v>
       </c>
       <c r="I3">
-        <v>0.25</v>
-      </c>
-      <c r="J3">
         <v>0.5</v>
       </c>
     </row>
@@ -519,12 +510,9 @@
         <v>good</v>
       </c>
       <c r="H4">
-        <v>18</v>
+        <v>0.18</v>
       </c>
       <c r="I4">
-        <v>0.18</v>
-      </c>
-      <c r="J4">
         <v>0.4</v>
       </c>
     </row>
@@ -551,25 +539,22 @@
         <v>great</v>
       </c>
       <c r="H5">
-        <v>12</v>
+        <v>0.12</v>
       </c>
       <c r="I5">
-        <v>0.12</v>
-      </c>
-      <c r="J5">
         <v>0.3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -709,58 +694,41 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>reclaimHours</v>
+        <v>captureChance</v>
       </c>
       <c r="B9" t="str">
         <v>float</v>
       </c>
       <c r="C9" t="str">
-        <v>不驻防被夺回的小时数</v>
+        <v>打赢后捕获守将的基础概率（0~1）</v>
       </c>
       <c r="D9" t="str">
-        <v>0=永久归你；如 12 表示占领后 12 小时内不留兵驻防则被中立/AI 夺回</v>
+        <v>如 0.25；品质越高的守将越难捕，deep 档调低</v>
       </c>
       <c r="E9" t="str">
-        <v>占领后若该城无驻军，经过此时长被重新设防夺走（0=永久，出生区/safe 档用 0）</v>
+        <v>到达战斗胜利后按此概率进入“捕获守将”面板（斩杀/招降/放生）；0=从不捕获</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>captureChance</v>
+        <v>recruitBaseRate</v>
       </c>
       <c r="B10" t="str">
         <v>float</v>
       </c>
       <c r="C10" t="str">
-        <v>打赢后捕获守将的基础概率（0~1）</v>
+        <v>招降基础成功率（0~1）</v>
       </c>
       <c r="D10" t="str">
-        <v>如 0.25；品质越高的守将越难捕，deep 档调低</v>
+        <v>如 0.5；后续好感度/羁绊/君主魅力系统会在此基础上加成</v>
       </c>
       <c r="E10" t="str">
-        <v>到达战斗胜利后按此概率进入“捕获守将”面板（斩杀/招降/放生）；0=从不捕获</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>recruitBaseRate</v>
-      </c>
-      <c r="B11" t="str">
-        <v>float</v>
-      </c>
-      <c r="C11" t="str">
-        <v>招降基础成功率（0~1）</v>
-      </c>
-      <c r="D11" t="str">
-        <v>如 0.5；后续好感度/羁绊/君主魅力系统会在此基础上加成</v>
-      </c>
-      <c r="E11" t="str">
         <v>捕获面板选“招降”时的基础成功率（当前无加成系统时即最终值）；失败守将流失</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>